<commit_message>
cái commit to chà bá vầy nè
</commit_message>
<xml_diff>
--- a/doc/DMC model.xlsx
+++ b/doc/DMC model.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Desktop\Phân tích DMC\Định giá\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\BCTC-CRAWLING PROJECT\Financial-Statement-Scraping\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{220524C7-F6EA-4076-A5A5-DEE9D5D4F904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620" firstSheet="2" activeTab="6"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BCTC du phong" sheetId="2" r:id="rId1"/>
@@ -24,22 +25,33 @@
   <externalReferences>
     <externalReference r:id="rId9"/>
   </externalReferences>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Tuan</author>
   </authors>
   <commentList>
-    <comment ref="B29" authorId="0" shapeId="0">
+    <comment ref="B29" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
       <text>
         <r>
           <rPr>
@@ -68,30 +80,12 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={000E9626-C71D-4368-8CAC-8972E9BF1CCD}</author>
     <author>VietHoang</author>
   </authors>
   <commentList>
-    <comment ref="B12" authorId="0" shapeId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Chú thích theo luồng]
-Phiên bản Excel của bạn cho phép bạn đọc chú thích theo luồng này; tuy nhiên, bất kỳ chỉnh sửa nào cho luồng cũng sẽ bị loại bỏ nếu mở tệp ở phiên bản Excel mới hơn. Tìm hiểu thêm: https://go.microsoft.com/fwlink/?linkid=870924
-Nhận xét:
-    HNX trai phieu</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A13" authorId="1" shapeId="0">
+    <comment ref="A13" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0600-000002000000}">
       <text>
         <r>
           <rPr>
@@ -1244,14 +1238,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="6">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="_-* #,##0.00\ _₫_-;\-* #,##0.00\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0\ _₫_-;\-* #,##0\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="168" formatCode="_-* #,##0.0\ _₫_-;\-* #,##0.0\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.00\ _₫_-;\-* #,##0.00\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0\ _₫_-;\-* #,##0\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="169" formatCode="_-* #,##0.0\ _₫_-;\-* #,##0.0\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
   </numFmts>
   <fonts count="16" x14ac:knownFonts="1">
     <font>
@@ -1613,27 +1607,27 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="197">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="5" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="5" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="5" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="5" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1641,120 +1635,120 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="5" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="5" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="2" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="8" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="8" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="7" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="9" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="10" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="9" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="10" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="7" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="8" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="9" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="10" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="7" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="9" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="10" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="8" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="9" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="10" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="9" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="10" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="7" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="8" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="9" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="10" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="8" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="9" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="10" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="43" fontId="0" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="11" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="167" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="168" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="12" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="12" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="37" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1767,7 +1761,7 @@
     <xf numFmtId="37" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="37" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="37" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="37" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="37" fontId="5" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1775,8 +1769,8 @@
     <xf numFmtId="37" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="37" fontId="8" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="37" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1786,12 +1780,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="13" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="37" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1800,23 +1794,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1833,12 +1821,6 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1851,7 +1833,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1860,13 +1842,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1875,14 +1857,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1918,7 +1912,6 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1995,7 +1988,6 @@
             <c:dispRSqr val="0"/>
             <c:dispEq val="1"/>
             <c:trendlineLbl>
-              <c:layout/>
               <c:numFmt formatCode="General" sourceLinked="0"/>
               <c:spPr>
                 <a:noFill/>
@@ -2690,7 +2682,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -4165,7 +4156,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -4277,7 +4267,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -4984,7 +4973,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -9744,7 +9732,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks/>
         </xdr:cNvGraphicFramePr>
@@ -9776,7 +9770,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks/>
         </xdr:cNvGraphicFramePr>
@@ -9808,7 +9808,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 3"/>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks/>
         </xdr:cNvGraphicFramePr>
@@ -9840,7 +9846,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Chart 4"/>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks/>
         </xdr:cNvGraphicFramePr>
@@ -9872,7 +9884,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="6" name="Chart 5"/>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000006000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks/>
         </xdr:cNvGraphicFramePr>
@@ -9904,7 +9922,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="7" name="Chart 6"/>
+        <xdr:cNvPr id="7" name="Chart 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000007000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks/>
         </xdr:cNvGraphicFramePr>
@@ -9925,7 +9949,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="HOME"/>
@@ -10366,7 +10390,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Trang_tính7"/>
   <dimension ref="A1:XFD328"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -38902,7 +38926,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Trang_tính6"/>
   <dimension ref="A1:K45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -39875,7 +39899,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Trang_tính2"/>
   <dimension ref="A1:K89"/>
   <sheetFormatPr defaultColWidth="20.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -40158,11 +40182,11 @@
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G9" s="2" t="str">
         <f>"&gt;="&amp;MIN(C8:F8)</f>
-        <v>&gt;=117.190353207675</v>
+        <v>&gt;=117,190353207675</v>
       </c>
       <c r="H9" s="99" t="str">
         <f>"&lt;"&amp;MIN(C8:F8)*10</f>
-        <v>&lt;1171.90353207675</v>
+        <v>&lt;1171,90353207675</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -40850,11 +40874,11 @@
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G31" s="2" t="str">
         <f>"&gt;="&amp;MIN(C30:F30)</f>
-        <v>&gt;=2.64303802463598</v>
+        <v>&gt;=2,64303802463598</v>
       </c>
       <c r="H31" s="99" t="str">
         <f>"&lt;"&amp;MIN(C30:F30)*10</f>
-        <v>&lt;26.4303802463598</v>
+        <v>&lt;26,4303802463598</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
@@ -41584,11 +41608,11 @@
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G56" s="2" t="str">
         <f>"&gt;="&amp;MIN(C55:F55)</f>
-        <v>&gt;=4.46740550554272</v>
+        <v>&gt;=4,46740550554272</v>
       </c>
       <c r="H56" s="99" t="str">
         <f>"&lt;"&amp;MIN(C55:F55)*10</f>
-        <v>&lt;44.6740550554272</v>
+        <v>&lt;44,6740550554272</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
@@ -42562,7 +42586,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Trang_tính3"/>
   <dimension ref="A1:L37"/>
   <sheetFormatPr defaultColWidth="20.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -43518,27 +43542,27 @@
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G37" s="2" t="str">
         <f>"&gt;="&amp;MIN(C36:F36)</f>
-        <v>&gt;=0.00960630492322467</v>
+        <v>&gt;=0,00960630492322467</v>
       </c>
       <c r="H37" s="99" t="str">
         <f>"&lt;"&amp;MIN(C36:F36)*10</f>
-        <v>&lt;0.0960630492322467</v>
+        <v>&lt;0,0960630492322467</v>
       </c>
       <c r="I37" s="2" t="str">
         <f>"&lt;="&amp;G36</f>
-        <v>&lt;=0.0190822927710484</v>
+        <v>&lt;=0,0190822927710484</v>
       </c>
       <c r="J37" s="2" t="str">
         <f>"&lt;="&amp;H36</f>
-        <v>&lt;=0.0157793435504106</v>
+        <v>&lt;=0,0157793435504106</v>
       </c>
       <c r="K37" s="2" t="str">
         <f>"&lt;="&amp;I36</f>
-        <v>&lt;=0.0157793435504106</v>
+        <v>&lt;=0,0157793435504106</v>
       </c>
       <c r="L37" s="2" t="str">
         <f>"&lt;="&amp;J36</f>
-        <v>&lt;=0.0157793435504106</v>
+        <v>&lt;=0,0157793435504106</v>
       </c>
     </row>
   </sheetData>
@@ -43547,7 +43571,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr codeName="Trang_tính4"/>
   <dimension ref="A1:K47"/>
   <sheetFormatPr defaultColWidth="20.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -44641,7 +44665,7 @@
         <v>2.9165769437420481</v>
       </c>
       <c r="H34" s="145">
-        <f t="shared" ref="G34:K34" si="10">IFERROR(H31/H26,0)</f>
+        <f t="shared" ref="H34:K34" si="10">IFERROR(H31/H26,0)</f>
         <v>3.0477979594544484</v>
       </c>
       <c r="I34" s="145">
@@ -45179,7 +45203,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Trang_tính5"/>
   <dimension ref="A1:K36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -46012,7 +46036,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr codeName="Trang_tính1"/>
   <dimension ref="A1:H61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -47220,10 +47244,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3" xr:uid="{00000000-0002-0000-0600-000000000000}">
       <formula1>"Best case, Base case, Worst case"</formula1>
     </dataValidation>
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="F2">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{00000000-0002-0000-0600-000001000000}">
       <formula1>"Tăng trưởng đều, Theo trend, Theo tăng trưởng quý"</formula1>
     </dataValidation>
   </dataValidations>
@@ -47234,7 +47258,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A2:P34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -47247,23 +47271,23 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="179" t="s">
+      <c r="A2" s="177" t="s">
         <v>157</v>
       </c>
-      <c r="B2" s="180" t="s">
+      <c r="B2" s="191" t="s">
         <v>158</v>
       </c>
-      <c r="C2" s="181"/>
-      <c r="D2" s="182" t="s">
+      <c r="C2" s="192"/>
+      <c r="D2" s="178" t="s">
         <v>159</v>
       </c>
-      <c r="E2" s="183" t="s">
+      <c r="E2" s="179" t="s">
         <v>160</v>
       </c>
-      <c r="F2" s="182" t="s">
+      <c r="F2" s="178" t="s">
         <v>161</v>
       </c>
-      <c r="G2" s="182" t="s">
+      <c r="G2" s="178" t="s">
         <v>162</v>
       </c>
       <c r="J2" s="21"/>
@@ -47278,12 +47302,12 @@
       </c>
       <c r="C3" s="170"/>
       <c r="D3" s="170"/>
-      <c r="E3" s="184"/>
+      <c r="E3" s="180"/>
       <c r="F3" s="170"/>
       <c r="G3" s="170"/>
     </row>
     <row r="4" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="185">
+      <c r="A4" s="181">
         <v>1</v>
       </c>
       <c r="B4" s="169" t="s">
@@ -47306,7 +47330,7 @@
       </c>
     </row>
     <row r="5" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="185">
+      <c r="A5" s="181">
         <v>2</v>
       </c>
       <c r="B5" s="169" t="s">
@@ -47329,7 +47353,7 @@
       </c>
     </row>
     <row r="6" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="185">
+      <c r="A6" s="181">
         <v>3</v>
       </c>
       <c r="B6" s="169" t="s">
@@ -47352,7 +47376,7 @@
       </c>
     </row>
     <row r="7" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="185">
+      <c r="A7" s="181">
         <v>4</v>
       </c>
       <c r="B7" s="169" t="s">
@@ -47379,7 +47403,7 @@
       <c r="A8" s="168" t="s">
         <v>165</v>
       </c>
-      <c r="B8" s="186" t="s">
+      <c r="B8" s="182" t="s">
         <v>166</v>
       </c>
       <c r="C8" s="170"/>
@@ -47395,13 +47419,13 @@
       <c r="P8" s="56"/>
     </row>
     <row r="9" spans="1:16" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="176">
+      <c r="A9" s="174">
         <v>1</v>
       </c>
-      <c r="B9" s="173" t="s">
+      <c r="B9" s="195" t="s">
         <v>167</v>
       </c>
-      <c r="C9" s="174"/>
+      <c r="C9" s="196"/>
       <c r="D9" s="166"/>
       <c r="E9" s="166">
         <f>TSCĐ!E21</f>
@@ -47422,12 +47446,12 @@
       <c r="A10" s="168" t="s">
         <v>168</v>
       </c>
-      <c r="B10" s="186" t="s">
+      <c r="B10" s="182" t="s">
         <v>77</v>
       </c>
       <c r="C10" s="170"/>
-      <c r="D10" s="184"/>
-      <c r="E10" s="184"/>
+      <c r="D10" s="180"/>
+      <c r="E10" s="180"/>
       <c r="F10" s="170"/>
       <c r="G10" s="170"/>
       <c r="K10" s="56"/>
@@ -47438,18 +47462,18 @@
       <c r="P10" s="56"/>
     </row>
     <row r="11" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="185">
+      <c r="A11" s="181">
         <v>1</v>
       </c>
       <c r="B11" s="169" t="s">
         <v>169</v>
       </c>
       <c r="C11" s="170"/>
-      <c r="D11" s="187">
+      <c r="D11" s="183">
         <f>TSCĐ!F36</f>
         <v>2.3974004568308546E-2</v>
       </c>
-      <c r="E11" s="187">
+      <c r="E11" s="183">
         <f>TSCĐ!G36</f>
         <v>1.9082292771048424E-2</v>
       </c>
@@ -47470,12 +47494,12 @@
       <c r="A12" s="168" t="s">
         <v>170</v>
       </c>
-      <c r="B12" s="186" t="s">
+      <c r="B12" s="182" t="s">
         <v>80</v>
       </c>
       <c r="C12" s="170"/>
-      <c r="D12" s="184"/>
-      <c r="E12" s="184"/>
+      <c r="D12" s="180"/>
+      <c r="E12" s="180"/>
       <c r="F12" s="170"/>
       <c r="G12" s="170"/>
       <c r="K12" s="56"/>
@@ -47486,18 +47510,18 @@
       <c r="P12" s="56"/>
     </row>
     <row r="13" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="188">
+      <c r="A13" s="184">
         <v>1</v>
       </c>
-      <c r="B13" s="189" t="s">
+      <c r="B13" s="185" t="s">
         <v>90</v>
       </c>
       <c r="C13" s="170"/>
-      <c r="D13" s="190">
+      <c r="D13" s="186">
         <f>'Vốn CSH'!F39</f>
         <v>0.37319756384295588</v>
       </c>
-      <c r="E13" s="190">
+      <c r="E13" s="186">
         <f>'Vốn CSH'!G39</f>
         <v>0.37634831631198745</v>
       </c>
@@ -47509,18 +47533,18 @@
       </c>
     </row>
     <row r="14" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="188">
+      <c r="A14" s="184">
         <v>2</v>
       </c>
-      <c r="B14" s="191" t="s">
+      <c r="B14" s="187" t="s">
         <v>86</v>
       </c>
       <c r="C14" s="170"/>
-      <c r="D14" s="190">
+      <c r="D14" s="186">
         <f>'Vốn CSH'!F34</f>
         <v>2.6308447584613726</v>
       </c>
-      <c r="E14" s="190">
+      <c r="E14" s="186">
         <f>'Vốn CSH'!G34</f>
         <v>2.9165769437420481</v>
       </c>
@@ -47532,18 +47556,18 @@
       </c>
     </row>
     <row r="15" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="188">
+      <c r="A15" s="184">
         <v>3</v>
       </c>
-      <c r="B15" s="191" t="s">
+      <c r="B15" s="187" t="s">
         <v>88</v>
       </c>
       <c r="C15" s="170"/>
-      <c r="D15" s="192">
+      <c r="D15" s="188">
         <f>'Vốn CSH'!F36</f>
         <v>3.0029506531857479E-2</v>
       </c>
-      <c r="E15" s="187">
+      <c r="E15" s="183">
         <f>'Vốn CSH'!G36</f>
         <v>3.0029506531857479E-2</v>
       </c>
@@ -47558,28 +47582,28 @@
       <c r="A16" s="168" t="s">
         <v>171</v>
       </c>
-      <c r="B16" s="186" t="s">
+      <c r="B16" s="182" t="s">
         <v>156</v>
       </c>
       <c r="C16" s="170"/>
-      <c r="D16" s="184"/>
-      <c r="E16" s="184"/>
+      <c r="D16" s="180"/>
+      <c r="E16" s="180"/>
       <c r="F16" s="170"/>
       <c r="G16" s="170"/>
     </row>
     <row r="17" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A17" s="175">
+      <c r="A17" s="173">
         <v>1</v>
       </c>
-      <c r="B17" s="177" t="s">
+      <c r="B17" s="175" t="s">
         <v>100</v>
       </c>
       <c r="C17" s="165"/>
-      <c r="D17" s="178">
+      <c r="D17" s="176">
         <f>'DT&amp;CP tài chính'!F19</f>
         <v>0</v>
       </c>
-      <c r="E17" s="178">
+      <c r="E17" s="176">
         <f>'DT&amp;CP tài chính'!G19</f>
         <v>4.2630604455403454E-2</v>
       </c>
@@ -47591,18 +47615,18 @@
       </c>
     </row>
     <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="185">
+      <c r="A18" s="181">
         <v>2</v>
       </c>
-      <c r="B18" s="193" t="s">
+      <c r="B18" s="189" t="s">
         <v>99</v>
       </c>
       <c r="C18" s="170"/>
-      <c r="D18" s="187">
+      <c r="D18" s="183">
         <f>'DT&amp;CP tài chính'!F16</f>
         <v>5.8018878202585659E-2</v>
       </c>
-      <c r="E18" s="187">
+      <c r="E18" s="183">
         <f>'DT&amp;CP tài chính'!G16</f>
         <v>5.8018878202585659E-2</v>
       </c>
@@ -47617,28 +47641,28 @@
       <c r="A19" s="168" t="s">
         <v>172</v>
       </c>
-      <c r="B19" s="186" t="s">
+      <c r="B19" s="182" t="s">
         <v>173</v>
       </c>
       <c r="C19" s="170"/>
-      <c r="D19" s="184"/>
-      <c r="E19" s="184"/>
+      <c r="D19" s="180"/>
+      <c r="E19" s="180"/>
       <c r="F19" s="170"/>
       <c r="G19" s="170"/>
     </row>
     <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="185">
+      <c r="A20" s="181">
         <v>1</v>
       </c>
-      <c r="B20" s="193" t="s">
+      <c r="B20" s="189" t="s">
         <v>174</v>
       </c>
       <c r="C20" s="170"/>
-      <c r="D20" s="187">
+      <c r="D20" s="183">
         <f>'DT&amp;CP tài chính'!E24</f>
         <v>0.02</v>
       </c>
-      <c r="E20" s="187">
+      <c r="E20" s="183">
         <f>'DT&amp;CP tài chính'!E24</f>
         <v>0.02</v>
       </c>
@@ -47650,18 +47674,18 @@
       </c>
     </row>
     <row r="21" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="185">
+      <c r="A21" s="181">
         <v>2</v>
       </c>
-      <c r="B21" s="193" t="s">
+      <c r="B21" s="189" t="s">
         <v>114</v>
       </c>
       <c r="C21" s="170"/>
-      <c r="D21" s="187">
+      <c r="D21" s="183">
         <f>'DT&amp;CP tài chính'!G32</f>
         <v>5.8018878202585659E-2</v>
       </c>
-      <c r="E21" s="187">
+      <c r="E21" s="183">
         <f>'DT&amp;CP tài chính'!G32</f>
         <v>5.8018878202585659E-2</v>
       </c>
@@ -47673,18 +47697,18 @@
       </c>
     </row>
     <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="185">
+      <c r="A22" s="181">
         <v>3</v>
       </c>
-      <c r="B22" s="193" t="s">
+      <c r="B22" s="189" t="s">
         <v>115</v>
       </c>
       <c r="C22" s="170"/>
-      <c r="D22" s="187">
+      <c r="D22" s="183">
         <f>'DT&amp;CP tài chính'!F33</f>
         <v>0</v>
       </c>
-      <c r="E22" s="187">
+      <c r="E22" s="183">
         <f>'DT&amp;CP tài chính'!G33</f>
         <v>0</v>
       </c>
@@ -47695,7 +47719,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="168" t="s">
         <v>175</v>
       </c>
@@ -47703,11 +47727,11 @@
         <v>176</v>
       </c>
       <c r="C23" s="170"/>
-      <c r="D23" s="187">
+      <c r="D23" s="183">
         <f>'Doanh thu'!F7</f>
         <v>6.0141875079662288E-2</v>
       </c>
-      <c r="E23" s="187">
+      <c r="E23" s="183">
         <f>'Doanh thu'!G7</f>
         <v>-2.5008231632909661E-2</v>
       </c>
@@ -47717,18 +47741,18 @@
       <c r="G23" s="170"/>
     </row>
     <row r="24" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A24" s="185">
+      <c r="A24" s="181">
         <v>1</v>
       </c>
-      <c r="B24" s="194" t="s">
+      <c r="B24" s="193" t="s">
         <v>355</v>
       </c>
-      <c r="C24" s="195"/>
-      <c r="D24" s="187">
+      <c r="C24" s="194"/>
+      <c r="D24" s="183">
         <f>'Doanh thu'!F11</f>
         <v>-5.0226380923634184E-2</v>
       </c>
-      <c r="E24" s="187">
+      <c r="E24" s="183">
         <f>'Doanh thu'!G11</f>
         <v>-0.2</v>
       </c>
@@ -47740,18 +47764,18 @@
       </c>
     </row>
     <row r="25" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A25" s="185">
+      <c r="A25" s="181">
         <v>2</v>
       </c>
-      <c r="B25" s="194" t="s">
+      <c r="B25" s="193" t="s">
         <v>356</v>
       </c>
-      <c r="C25" s="195"/>
-      <c r="D25" s="187">
+      <c r="C25" s="194"/>
+      <c r="D25" s="183">
         <f>'Doanh thu'!F14</f>
         <v>0.62757278534775685</v>
       </c>
-      <c r="E25" s="187">
+      <c r="E25" s="183">
         <f>'Doanh thu'!G14</f>
         <v>0.5</v>
       </c>
@@ -47770,21 +47794,21 @@
         <v>116</v>
       </c>
       <c r="C26" s="170"/>
-      <c r="D26" s="184"/>
-      <c r="E26" s="184"/>
+      <c r="D26" s="180"/>
+      <c r="E26" s="180"/>
       <c r="F26" s="170"/>
       <c r="G26" s="170"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="185">
+      <c r="A27" s="181">
         <v>1</v>
       </c>
-      <c r="B27" s="193" t="s">
+      <c r="B27" s="189" t="s">
         <v>357</v>
       </c>
       <c r="C27" s="170"/>
-      <c r="D27" s="187"/>
-      <c r="E27" s="187">
+      <c r="D27" s="183"/>
+      <c r="E27" s="183">
         <v>1</v>
       </c>
       <c r="F27" s="170"/>
@@ -47793,15 +47817,15 @@
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="185">
+      <c r="A28" s="181">
         <v>2</v>
       </c>
-      <c r="B28" s="193" t="s">
+      <c r="B28" s="189" t="s">
         <v>178</v>
       </c>
       <c r="C28" s="170"/>
-      <c r="D28" s="187"/>
-      <c r="E28" s="196">
+      <c r="D28" s="183"/>
+      <c r="E28" s="190">
         <f>'Định giá'!B25</f>
         <v>2.5000000000000001E-2</v>
       </c>
@@ -47818,22 +47842,22 @@
         <v>180</v>
       </c>
       <c r="C29" s="170"/>
-      <c r="D29" s="184"/>
-      <c r="E29" s="184"/>
+      <c r="D29" s="180"/>
+      <c r="E29" s="180"/>
       <c r="F29" s="170"/>
       <c r="G29" s="170"/>
     </row>
     <row r="30" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="193"/>
-      <c r="B30" s="193" t="s">
+      <c r="A30" s="189"/>
+      <c r="B30" s="189" t="s">
         <v>3</v>
       </c>
       <c r="C30" s="170"/>
-      <c r="D30" s="187">
+      <c r="D30" s="183">
         <f>'BCTC du phong'!G20</f>
         <v>0.18694946771385557</v>
       </c>
-      <c r="E30" s="187">
+      <c r="E30" s="183">
         <f>'BCTC du phong'!H20</f>
         <v>0.18694946771385557</v>
       </c>
@@ -47845,16 +47869,16 @@
       </c>
     </row>
     <row r="31" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" s="193"/>
-      <c r="B31" s="193" t="s">
+      <c r="A31" s="189"/>
+      <c r="B31" s="189" t="s">
         <v>181</v>
       </c>
       <c r="C31" s="170"/>
-      <c r="D31" s="187">
+      <c r="D31" s="183">
         <f>'BCTC du phong'!G24</f>
         <v>0</v>
       </c>
-      <c r="E31" s="187">
+      <c r="E31" s="183">
         <f>'BCTC du phong'!H24</f>
         <v>0</v>
       </c>

</xml_diff>